<commit_message>
Refresh Sleeper data (2026-08-13)
</commit_message>
<xml_diff>
--- a/output/2026/rosters-pre-draft-2026-ffl.xlsx
+++ b/output/2026/rosters-pre-draft-2026-ffl.xlsx
@@ -304,9 +304,9 @@
           <t>Chase, Ja'Marr CIN WR</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Cook, James BUF RB</t>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Bowers, Brock LV TE</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -358,7 +358,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Brown, Chase CIN RB</t>
+          <t>Cook, James BUF RB</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -394,9 +394,9 @@
           <t>Taylor, Jonathan IND RB</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Bowers, Brock LV TE</t>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Nix, Bo DEN QB</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -404,7 +404,11 @@
           <t>McBride, Trey ARI TE</t>
         </is>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Brown, Chase CIN RB</t>
+        </is>
+      </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Nacua, Puka LAR WR</t>
@@ -438,9 +442,9 @@
           <t>Wilson, Garrett NYJ WR</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Nix, Bo DEN QB</t>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Jacobs, Josh GB RB</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -482,9 +486,9 @@
           <t>Higgins, Tee CIN WR</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Jacobs, Josh GB RB</t>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Herbert, Justin LAC QB</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -506,11 +510,7 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Herbert, Justin LAC QB</t>
-        </is>
-      </c>
+      <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="5" t="inlineStr">
@@ -840,17 +840,17 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>Shough, Tyler NO QB</t>
+          <t>Stafford, Matthew LAR QB</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>Godwin, Chris TB WR</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Stafford, Matthew LAR QB</t>
+          <t>Olave, Chris NO WR</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Reed, Jayden GB WR</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -880,9 +880,9 @@
           <t>Jeudy, Jerry CLE WR</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Olave, Chris NO WR</t>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Bigsby, Tank PHI RB</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -895,14 +895,14 @@
           <t>Fannin, Harold CLE TE</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Sanders, Shedeur CLE QB</t>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Godwin, Chris TB WR</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Reed, Jayden GB WR</t>
+          <t>Allen, Keenan FA WR</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -932,9 +932,9 @@
           <t>Darnold, Sam SEA QB</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Bigsby, Tank PHI RB</t>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Burden, Luther CHI WR</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -947,14 +947,10 @@
           <t>Higgins, Jayden HOU WR</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Davis, Malik DAL RB</t>
-        </is>
-      </c>
+      <c r="H20" s="2"/>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Allen, Keenan FA WR</t>
+          <t>Pierce, Alec IND WR</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -984,9 +980,9 @@
           <t>Aiyuk, Brandon SF WR</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Burden, Luther CHI WR</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Gainwell, Kenny TB RB</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -999,14 +995,10 @@
           <t>Allgeier, Tyler ARI RB</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Hunt, Kareem FA RB</t>
-        </is>
-      </c>
+      <c r="H21" s="2"/>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Pierce, Alec IND WR</t>
+          <t>Watson, Christian GB WR</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1036,9 +1028,9 @@
           <t>Dowdle, Rico PIT RB</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Gainwell, Kenny TB RB</t>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>TeSlaa, Isaac DET WR</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -1046,19 +1038,15 @@
           <t>Chiefs, Kansas City KC DEF</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Carter, Michael TEN RB</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>Johnson, Juwan NO TE</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>Watson, Christian GB WR</t>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Shough, Tyler NO QB</t>
+        </is>
+      </c>
+      <c r="H22" s="2"/>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Parkinson, Colby LAR TE</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -1088,9 +1076,9 @@
           <t>Knight, Zonovan ARI RB</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>TeSlaa, Isaac DET WR</t>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Lions, Detroit DET DEF</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1103,14 +1091,10 @@
           <t>Wilson, Emanuel SEA RB</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>Seahawks, Seattle SEA DEF</t>
-        </is>
-      </c>
+      <c r="H23" s="2"/>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Parkinson, Colby LAR TE</t>
+          <t>Schultz, Dalton HOU TE</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -1140,9 +1124,9 @@
           <t>Vikings, Minnesota MIN DEF</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Lions, Detroit DET DEF</t>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Aubrey, Brandon DAL K</t>
         </is>
       </c>
       <c r="F24" s="2"/>
@@ -1151,14 +1135,10 @@
           <t>Robinson, Wan'Dale TEN WR</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>Fairbairn, Ka'imi HOU K</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>Schultz, Dalton HOU TE</t>
+      <c r="H24" s="2"/>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>Steelers, Pittsburgh PIT DEF</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
@@ -1188,11 +1168,7 @@
           <t>Lutz, Wil DEN K</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>Aubrey, Brandon DAL K</t>
-        </is>
-      </c>
+      <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="5" t="inlineStr">
         <is>
@@ -1200,9 +1176,9 @@
         </is>
       </c>
       <c r="H25" s="2"/>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>Steelers, Pittsburgh PIT DEF</t>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Little, Cam JAX K</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -1218,9 +1194,9 @@
           <t>Boswell, Chris PIT K</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Jaguars, Jacksonville JAX DEF</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Loop, Tyler BAL K</t>
         </is>
       </c>
       <c r="D26" s="2"/>
@@ -1232,11 +1208,7 @@
         </is>
       </c>
       <c r="H26" s="2"/>
-      <c r="I26" s="8" t="inlineStr">
-        <is>
-          <t>Little, Cam JAX K</t>
-        </is>
-      </c>
+      <c r="I26" s="2"/>
       <c r="J26" s="7" t="inlineStr">
         <is>
           <t>Saints, New Orleans NO DEF</t>
@@ -1246,11 +1218,7 @@
     <row r="27">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Loop, Tyler BAL K</t>
-        </is>
-      </c>
+      <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -1278,7 +1246,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Data retrieved Aug 12, 2026, 5:01 AM PT</t>
+          <t>Data retrieved Aug 12, 2026, 10:14 PM PT</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1261,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1415,17 +1383,17 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Visalia Viagra Vipers</t>
+          <t>Vancouver Moose Drool</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Easton Evil Empire</t>
+          <t>Kingsburg Killaz</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>Nov 12, 2025</t>
+          <t>Aug 12, 2026</t>
         </is>
       </c>
     </row>
@@ -1436,21 +1404,71 @@
         </is>
       </c>
       <c r="B6" s="15">
+        <v>5</v>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Visalia Viagra Vipers</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Easton Evil Empire</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Nov 12, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
         <v>6</v>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Vancouver Moose Drool</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Sanger Squatty Pottys</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Nov 12, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <v>7</v>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Sanger Squatty Pottys</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Dinkey Creek Dirt Clods</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Aug 12, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh Sleeper data (2026-08-14)
</commit_message>
<xml_diff>
--- a/output/2026/rosters-pre-draft-2026-ffl.xlsx
+++ b/output/2026/rosters-pre-draft-2026-ffl.xlsx
@@ -279,7 +279,7 @@
           <t>Jefferson, Justin MIN WR</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>McCaffrey, Christian SF RB</t>
         </is>
@@ -823,7 +823,7 @@
           <t>Tagovailoa, Tua ATL QB</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Skattebo, Cam NYG RB</t>
         </is>
@@ -875,9 +875,9 @@
           <t>Dart, Jaxson NYG QB</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Jeudy, Jerry CLE WR</t>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Darnold, Sam SEA QB</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -927,9 +927,9 @@
           <t>Rivers, Philip FA QB</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Darnold, Sam SEA QB</t>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Jeudy, Jerry CLE WR</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1246,7 +1246,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Data retrieved Aug 13, 2026, 5:02 AM PT</t>
+          <t>Data retrieved Aug 14, 2026, 4:59 AM PT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh Sleeper data (2026-08-19)
</commit_message>
<xml_diff>
--- a/output/2026/rosters-pre-draft-2026-ffl.xlsx
+++ b/output/2026/rosters-pre-draft-2026-ffl.xlsx
@@ -264,7 +264,7 @@
       <c r="J2" s="10"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Burrow, Joe CIN QB</t>
         </is>
@@ -536,61 +536,61 @@
       <c r="J9" s="11"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Smith, DeVonta PHI WR</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>McCarthy, J.J. MIN QB</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Worthy, Xavier KC WR</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Harvey, RJ DEN RB</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Williams, Caleb CHI QB</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Purdy, Brock SF QB</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Kamara, Alvin NO RB</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Maye, Drake NE QB</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Goff, Jared DET QB</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Pickens, George DAL WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Swift, D'Andre CHI RB</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>McCarthy, J.J. MIN QB</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Worthy, Xavier KC WR</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Harvey, RJ DEN RB</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Williams, Caleb CHI QB</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Purdy, Brock SF QB</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Kamara, Alvin NO RB</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>Maye, Drake NE QB</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Goff, Jared DET QB</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>Pickens, George DAL WR</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Smith, DeVonta PHI WR</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -808,9 +808,9 @@
       <c r="J17" s="12"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Jennings, Jauan MIN WR</t>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Shakir, Khalil BUF WR</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -862,7 +862,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Shakir, Khalil BUF WR</t>
+          <t>Jennings, Jauan MIN WR</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Allen, Keenan FA WR</t>
+          <t>Allen, Keenan IND WR</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -1246,7 +1246,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Data retrieved Aug 18, 2026, 4:43 AM PT</t>
+          <t>Data retrieved Aug 19, 2026, 4:43 AM PT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh Sleeper data (2026-08-20)
</commit_message>
<xml_diff>
--- a/output/2026/rosters-pre-draft-2026-ffl.xlsx
+++ b/output/2026/rosters-pre-draft-2026-ffl.xlsx
@@ -269,9 +269,9 @@
           <t>Burrow, Joe CIN QB</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Daniels, Jayden WAS QB</t>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Smith-Njigba, Jaxon SEA WR</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -309,9 +309,9 @@
           <t>Bowers, Brock LV TE</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Hurts, Jalen PHI QB</t>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Nacua, Puka LAR WR</t>
         </is>
       </c>
     </row>
@@ -321,9 +321,9 @@
           <t>St. Brown, Amon-Ra DET WR</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Smith-Njigba, Jaxon SEA WR</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Daniels, Jayden WAS QB</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -361,9 +361,9 @@
           <t>Cook, James BUF RB</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Henry, Derrick BAL RB</t>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Hurts, Jalen PHI QB</t>
         </is>
       </c>
     </row>
@@ -409,9 +409,9 @@
           <t>Brown, Chase CIN RB</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Nacua, Puka LAR WR</t>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Henry, Derrick BAL RB</t>
         </is>
       </c>
     </row>
@@ -541,9 +541,9 @@
           <t>Smith, DeVonta PHI WR</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>McCarthy, J.J. MIN QB</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Egbuka, Emeka TB WR</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -581,7 +581,7 @@
           <t>Goff, Jared DET QB</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>Pickens, George DAL WR</t>
         </is>
@@ -593,9 +593,9 @@
           <t>Swift, D'Andre CHI RB</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Odunze, Rome CHI WR</t>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>McCarthy, J.J. MIN QB</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Williams, Jameson DET WR</t>
+          <t>Odunze, Rome CHI WR</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -681,9 +681,9 @@
           <t>Warren, Jaylen PIT RB</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Charbonnet, Zach SEA RB</t>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Williams, Jameson DET WR</t>
         </is>
       </c>
       <c r="C13" s="2"/>
@@ -717,9 +717,9 @@
     </row>
     <row r="14">
       <c r="A14" s="2"/>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Andrews, Mark BAL TE</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Charbonnet, Zach SEA RB</t>
         </is>
       </c>
       <c r="C14" s="2"/>
@@ -749,9 +749,9 @@
     </row>
     <row r="15">
       <c r="A15" s="2"/>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Egbuka, Emeka TB WR</t>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Andrews, Mark BAL TE</t>
         </is>
       </c>
       <c r="C15" s="2"/>
@@ -813,7 +813,7 @@
           <t>Shakir, Khalil BUF WR</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Lawrence, Trevor JAX QB</t>
         </is>
@@ -853,9 +853,9 @@
           <t>Reed, Jayden GB WR</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Stevenson, Rhamondre NE RB</t>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Brissett, Jacoby ARI QB</t>
         </is>
       </c>
     </row>
@@ -905,9 +905,9 @@
           <t>Allen, Keenan IND WR</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Pittman, Michael PIT WR</t>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Stevenson, Rhamondre NE RB</t>
         </is>
       </c>
     </row>
@@ -953,9 +953,9 @@
           <t>Pierce, Alec IND WR</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Brissett, Jacoby ARI QB</t>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Pittman, Michael PIT WR</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Data retrieved Aug 19, 2026, 9:47 AM PT</t>
+          <t>Data retrieved Aug 19, 2026, 8:55 PM PT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh Sleeper data (2026-08-21)
</commit_message>
<xml_diff>
--- a/output/2026/rosters-pre-draft-2026-ffl.xlsx
+++ b/output/2026/rosters-pre-draft-2026-ffl.xlsx
@@ -274,7 +274,7 @@
           <t>Smith-Njigba, Jaxon SEA WR</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Jefferson, Justin MIN WR</t>
         </is>
@@ -304,7 +304,7 @@
           <t>Chase, Ja'Marr CIN WR</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Bowers, Brock LV TE</t>
         </is>
@@ -546,9 +546,9 @@
           <t>Egbuka, Emeka TB WR</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Worthy, Xavier KC WR</t>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Rice, Rashee KC WR</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -576,9 +576,9 @@
           <t>Maye, Drake NE QB</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Goff, Jared DET QB</t>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>McMillan, Tetairoa CAR WR</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Rice, Rashee KC WR</t>
+          <t>Worthy, Xavier KC WR</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -624,9 +624,9 @@
           <t>McLaurin, Terry WAS WR</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Pollard, Tony TEN RB</t>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Goff, Jared DET QB</t>
         </is>
       </c>
       <c r="J11" s="2"/>
@@ -668,9 +668,9 @@
           <t>Diggs, Stefon WAS WR</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>McMillan, Tetairoa CAR WR</t>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Pollard, Tony TEN RB</t>
         </is>
       </c>
       <c r="J12" s="2"/>
@@ -818,9 +818,9 @@
           <t>Lawrence, Trevor JAX QB</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Tagovailoa, Tua ATL QB</t>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Dart, Jaxson NYG QB</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -848,9 +848,9 @@
           <t>Olave, Chris NO WR</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>Reed, Jayden GB WR</t>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Watson, Christian GB WR</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Dart, Jaxson NYG QB</t>
+          <t>Tagovailoa, Tua ATL QB</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Allen, Keenan IND WR</t>
+          <t>Reed, Jayden GB WR</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -950,7 +950,7 @@
       <c r="H20" s="2"/>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Pierce, Alec IND WR</t>
+          <t>Allen, Keenan IND WR</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
@@ -998,7 +998,7 @@
       <c r="H21" s="2"/>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Watson, Christian GB WR</t>
+          <t>Pierce, Alec IND WR</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1246,7 +1246,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Data retrieved Aug 21, 2026, 4:45 AM PT</t>
+          <t>Data retrieved Aug 21, 2026, 11:19 AM PT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh Sleeper data (2026-08-27)
</commit_message>
<xml_diff>
--- a/output/2026/rosters-pre-draft-2026-ffl.xlsx
+++ b/output/2026/rosters-pre-draft-2026-ffl.xlsx
@@ -892,7 +892,7 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Fannin, Harold CLE TE</t>
+          <t>Shough, Tyler NO QB</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1038,9 +1038,9 @@
           <t>Chiefs, Kansas City KC DEF</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Shough, Tyler NO QB</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Wilson, Emanuel SEA RB</t>
         </is>
       </c>
       <c r="H22" s="2"/>
@@ -1086,9 +1086,9 @@
           <t>Pineiro, Eddy SF K</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Wilson, Emanuel SEA RB</t>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Robinson, Wan'Dale TEN WR</t>
         </is>
       </c>
       <c r="H23" s="2"/>
@@ -1132,7 +1132,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Robinson, Wan'Dale TEN WR</t>
+          <t>Slayton, Darius NYG WR</t>
         </is>
       </c>
       <c r="H24" s="2"/>
@@ -1170,9 +1170,9 @@
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Slayton, Darius NYG WR</t>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Fannin, Harold CLE TE</t>
         </is>
       </c>
       <c r="H25" s="2"/>
@@ -1246,7 +1246,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Data retrieved Aug 26, 2026, 4:47 AM PT</t>
+          <t>Data retrieved Aug 27, 2026, 11:37 AM PT</t>
         </is>
       </c>
     </row>

</xml_diff>